<commit_message>
change xlr_double name to xlr_numeric, and changed its implementation to reflect this. I also added that it supports scientific notation, this has been added to test. Also fixed an issue with column widths, so now they look better.
</commit_message>
<xml_diff>
--- a/tests/testthat/_output_excel_snaps/data_to_worksheet.xlsx
+++ b/tests/testthat/_output_excel_snaps/data_to_worksheet.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">mpg</t>
   </si>
@@ -47,6 +47,9 @@
     <t xml:space="preserve">carb</t>
   </si>
   <si>
+    <t xml:space="preserve">scientific</t>
+  </si>
+  <si>
     <t xml:space="preserve">test</t>
   </si>
 </sst>
@@ -54,7 +57,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="0"/>
@@ -65,6 +68,7 @@
     <numFmt numFmtId="172" formatCode="0.00"/>
     <numFmt numFmtId="173" formatCode="0.00"/>
     <numFmt numFmtId="174" formatCode="0.00"/>
+    <numFmt numFmtId="175" formatCode="0.00E+00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -100,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -133,6 +137,9 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="174" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="175" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -459,6 +466,9 @@
       <c r="K2" t="s">
         <v>10</v>
       </c>
+      <c r="L2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -483,7 +493,7 @@
         <v>16.46</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I3" s="9" t="n">
         <v>1</v>
@@ -493,6 +503,9 @@
       </c>
       <c r="K3" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>16.46</v>
       </c>
     </row>
     <row r="4">
@@ -518,7 +531,7 @@
         <v>17.02</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I4" s="9" t="n">
         <v>1</v>
@@ -528,6 +541,9 @@
       </c>
       <c r="K4" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>17.02</v>
       </c>
     </row>
     <row r="5">
@@ -553,7 +569,7 @@
         <v>18.61</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I5" s="9" t="n">
         <v>1</v>
@@ -563,6 +579,9 @@
       </c>
       <c r="K5" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>18.61</v>
       </c>
     </row>
     <row r="6">
@@ -588,7 +607,7 @@
         <v>19.44</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I6" s="9" t="n">
         <v>0</v>
@@ -598,6 +617,9 @@
       </c>
       <c r="K6" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>19.44</v>
       </c>
     </row>
     <row r="7">
@@ -623,7 +645,7 @@
         <v>17.02</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I7" s="9" t="n">
         <v>0</v>
@@ -633,6 +655,9 @@
       </c>
       <c r="K7" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L7" s="12" t="n">
+        <v>17.02</v>
       </c>
     </row>
     <row r="8">
@@ -658,7 +683,7 @@
         <v>20.22</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I8" s="9" t="n">
         <v>0</v>
@@ -668,6 +693,9 @@
       </c>
       <c r="K8" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L8" s="12" t="n">
+        <v>20.22</v>
       </c>
     </row>
     <row r="9">
@@ -693,7 +721,7 @@
         <v>15.84</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I9" s="9" t="n">
         <v>0</v>
@@ -703,6 +731,9 @@
       </c>
       <c r="K9" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>15.84</v>
       </c>
     </row>
     <row r="10">
@@ -728,7 +759,7 @@
         <v>20</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I10" s="9" t="n">
         <v>0</v>
@@ -738,6 +769,9 @@
       </c>
       <c r="K10" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -763,7 +797,7 @@
         <v>22.9</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I11" s="9" t="n">
         <v>0</v>
@@ -773,6 +807,9 @@
       </c>
       <c r="K11" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>22.9</v>
       </c>
     </row>
     <row r="12">
@@ -798,7 +835,7 @@
         <v>18.3</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I12" s="9" t="n">
         <v>0</v>
@@ -808,6 +845,9 @@
       </c>
       <c r="K12" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>18.3</v>
       </c>
     </row>
     <row r="13">
@@ -833,7 +873,7 @@
         <v>18.9</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I13" s="9" t="n">
         <v>0</v>
@@ -843,6 +883,9 @@
       </c>
       <c r="K13" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>18.9</v>
       </c>
     </row>
     <row r="14">
@@ -868,7 +911,7 @@
         <v>17.4</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I14" s="9" t="n">
         <v>0</v>
@@ -878,6 +921,9 @@
       </c>
       <c r="K14" s="11" t="n">
         <v>3</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>17.4</v>
       </c>
     </row>
     <row r="15">
@@ -903,7 +949,7 @@
         <v>17.6</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I15" s="9" t="n">
         <v>0</v>
@@ -913,6 +959,9 @@
       </c>
       <c r="K15" s="11" t="n">
         <v>3</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>17.6</v>
       </c>
     </row>
     <row r="16">
@@ -938,7 +987,7 @@
         <v>18</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I16" s="9" t="n">
         <v>0</v>
@@ -948,6 +997,9 @@
       </c>
       <c r="K16" s="11" t="n">
         <v>3</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="17">
@@ -973,7 +1025,7 @@
         <v>17.98</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I17" s="9" t="n">
         <v>0</v>
@@ -983,6 +1035,9 @@
       </c>
       <c r="K17" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>17.98</v>
       </c>
     </row>
     <row r="18">
@@ -1008,7 +1063,7 @@
         <v>17.82</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I18" s="9" t="n">
         <v>0</v>
@@ -1018,6 +1073,9 @@
       </c>
       <c r="K18" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>17.82</v>
       </c>
     </row>
     <row r="19">
@@ -1043,7 +1101,7 @@
         <v>17.42</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I19" s="9" t="n">
         <v>0</v>
@@ -1053,6 +1111,9 @@
       </c>
       <c r="K19" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L19" s="12" t="n">
+        <v>17.42</v>
       </c>
     </row>
     <row r="20">
@@ -1078,7 +1139,7 @@
         <v>19.47</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I20" s="9" t="n">
         <v>1</v>
@@ -1088,6 +1149,9 @@
       </c>
       <c r="K20" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>19.47</v>
       </c>
     </row>
     <row r="21">
@@ -1113,7 +1177,7 @@
         <v>18.52</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I21" s="9" t="n">
         <v>1</v>
@@ -1123,6 +1187,9 @@
       </c>
       <c r="K21" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>18.52</v>
       </c>
     </row>
     <row r="22">
@@ -1148,7 +1215,7 @@
         <v>19.9</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I22" s="9" t="n">
         <v>1</v>
@@ -1158,6 +1225,9 @@
       </c>
       <c r="K22" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>19.9</v>
       </c>
     </row>
     <row r="23">
@@ -1183,7 +1253,7 @@
         <v>20.01</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I23" s="9" t="n">
         <v>0</v>
@@ -1193,6 +1263,9 @@
       </c>
       <c r="K23" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>20.01</v>
       </c>
     </row>
     <row r="24">
@@ -1218,7 +1291,7 @@
         <v>16.87</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I24" s="9" t="n">
         <v>0</v>
@@ -1228,6 +1301,9 @@
       </c>
       <c r="K24" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>16.87</v>
       </c>
     </row>
     <row r="25">
@@ -1253,7 +1329,7 @@
         <v>17.3</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I25" s="9" t="n">
         <v>0</v>
@@ -1263,6 +1339,9 @@
       </c>
       <c r="K25" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L25" s="12" t="n">
+        <v>17.3</v>
       </c>
     </row>
     <row r="26">
@@ -1288,7 +1367,7 @@
         <v>15.41</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I26" s="9" t="n">
         <v>0</v>
@@ -1298,6 +1377,9 @@
       </c>
       <c r="K26" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L26" s="12" t="n">
+        <v>15.41</v>
       </c>
     </row>
     <row r="27">
@@ -1323,7 +1405,7 @@
         <v>17.05</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I27" s="9" t="n">
         <v>0</v>
@@ -1333,6 +1415,9 @@
       </c>
       <c r="K27" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>17.05</v>
       </c>
     </row>
     <row r="28">
@@ -1358,7 +1443,7 @@
         <v>18.9</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I28" s="9" t="n">
         <v>1</v>
@@ -1368,6 +1453,9 @@
       </c>
       <c r="K28" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>18.9</v>
       </c>
     </row>
     <row r="29">
@@ -1393,7 +1481,7 @@
         <v>16.7</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I29" s="9" t="n">
         <v>1</v>
@@ -1403,6 +1491,9 @@
       </c>
       <c r="K29" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>16.7</v>
       </c>
     </row>
     <row r="30">
@@ -1428,7 +1519,7 @@
         <v>16.9</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I30" s="9" t="n">
         <v>1</v>
@@ -1438,6 +1529,9 @@
       </c>
       <c r="K30" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L30" s="12" t="n">
+        <v>16.9</v>
       </c>
     </row>
     <row r="31">
@@ -1463,7 +1557,7 @@
         <v>14.5</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I31" s="9" t="n">
         <v>1</v>
@@ -1473,6 +1567,9 @@
       </c>
       <c r="K31" s="11" t="n">
         <v>4</v>
+      </c>
+      <c r="L31" s="12" t="n">
+        <v>14.5</v>
       </c>
     </row>
     <row r="32">
@@ -1498,7 +1595,7 @@
         <v>15.5</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I32" s="9" t="n">
         <v>1</v>
@@ -1508,6 +1605,9 @@
       </c>
       <c r="K32" s="11" t="n">
         <v>6</v>
+      </c>
+      <c r="L32" s="12" t="n">
+        <v>15.5</v>
       </c>
     </row>
     <row r="33">
@@ -1533,7 +1633,7 @@
         <v>14.6</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I33" s="9" t="n">
         <v>1</v>
@@ -1543,6 +1643,9 @@
       </c>
       <c r="K33" s="11" t="n">
         <v>8</v>
+      </c>
+      <c r="L33" s="12" t="n">
+        <v>14.6</v>
       </c>
     </row>
     <row r="34">
@@ -1568,7 +1671,7 @@
         <v>18.6</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I34" s="9" t="n">
         <v>1</v>
@@ -1578,6 +1681,9 @@
       </c>
       <c r="K34" s="11" t="n">
         <v>2</v>
+      </c>
+      <c r="L34" s="12" t="n">
+        <v>18.6</v>
       </c>
     </row>
     <row r="35">
@@ -1592,6 +1698,7 @@
       <c r="I35" s="9"/>
       <c r="J35" s="10"/>
       <c r="K35" s="11"/>
+      <c r="L35" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added a new format, xlr_format_numeric, which has different default values to use with numeric types. Updated the types to use this new format.
</commit_message>
<xml_diff>
--- a/tests/testthat/_output_excel_snaps/data_to_worksheet.xlsx
+++ b/tests/testthat/_output_excel_snaps/data_to_worksheet.xlsx
@@ -113,16 +113,16 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -140,7 +140,7 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="175" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="right" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>

<commit_message>
fixed a bug where when using write_xlsx() was not writing factors correctly. This would have been an issue for a number of different types.
</commit_message>
<xml_diff>
--- a/tests/testthat/_output_excel_snaps/data_to_worksheet.xlsx
+++ b/tests/testthat/_output_excel_snaps/data_to_worksheet.xlsx
@@ -12,63 +12,62 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
-    <t xml:space="preserve">mpg</t>
+    <t xml:space="preserve">test_r_numeric</t>
   </si>
   <si>
-    <t xml:space="preserve">cyl</t>
+    <t xml:space="preserve">test_r_integer</t>
   </si>
   <si>
-    <t xml:space="preserve">disp</t>
+    <t xml:space="preserve">test_xlr_numeric</t>
   </si>
   <si>
-    <t xml:space="preserve">hp</t>
+    <t xml:space="preserve">test_xlr_vector</t>
   </si>
   <si>
-    <t xml:space="preserve">drat</t>
+    <t xml:space="preserve">test_xlr_numeric.1</t>
   </si>
   <si>
-    <t xml:space="preserve">wt</t>
+    <t xml:space="preserve">test_xlr_percent</t>
   </si>
   <si>
-    <t xml:space="preserve">qsec</t>
+    <t xml:space="preserve">test_r_char</t>
   </si>
   <si>
-    <t xml:space="preserve">vs</t>
+    <t xml:space="preserve">test_xlr_scientific</t>
   </si>
   <si>
-    <t xml:space="preserve">am</t>
+    <t xml:space="preserve">test_r_factor</t>
   </si>
   <si>
-    <t xml:space="preserve">gear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">scientific</t>
+    <t xml:space="preserve">test_r_complex</t>
   </si>
   <si>
     <t xml:space="preserve">test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1+1i</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="11">
+  <numFmts count="7">
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="0"/>
     <numFmt numFmtId="168" formatCode="0.00"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
     <numFmt numFmtId="170" formatCode="0.00%"/>
-    <numFmt numFmtId="171" formatCode="0.00"/>
-    <numFmt numFmtId="172" formatCode="0.00"/>
-    <numFmt numFmtId="173" formatCode="0.00"/>
-    <numFmt numFmtId="174" formatCode="0.00"/>
-    <numFmt numFmtId="175" formatCode="0.00E+00"/>
+    <numFmt numFmtId="171" formatCode="0.00E+00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -104,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -124,22 +123,10 @@
     <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="172" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="173" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="174" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="175" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -463,12 +450,6 @@
       <c r="J2" t="s">
         <v>9</v>
       </c>
-      <c r="K2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L2" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -489,23 +470,17 @@
       <c r="F3" s="6" t="n">
         <v>2.62</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="G3" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="8" t="n">
         <v>16.46</v>
       </c>
-      <c r="H3" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K3" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>16.46</v>
+      <c r="I3" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -527,23 +502,17 @@
       <c r="F4" s="6" t="n">
         <v>2.875</v>
       </c>
-      <c r="G4" s="7" t="n">
+      <c r="G4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="8" t="n">
         <v>17.02</v>
       </c>
-      <c r="H4" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K4" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>17.02</v>
+      <c r="I4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -565,23 +534,17 @@
       <c r="F5" s="6" t="n">
         <v>2.32</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="8" t="n">
         <v>18.61</v>
       </c>
-      <c r="H5" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>18.61</v>
+      <c r="I5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -603,23 +566,17 @@
       <c r="F6" s="6" t="n">
         <v>3.215</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="8" t="n">
         <v>19.44</v>
       </c>
-      <c r="H6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K6" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>19.44</v>
+      <c r="I6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -641,23 +598,17 @@
       <c r="F7" s="6" t="n">
         <v>3.44</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="8" t="n">
         <v>17.02</v>
       </c>
-      <c r="H7" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L7" s="12" t="n">
-        <v>17.02</v>
+      <c r="I7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -679,23 +630,17 @@
       <c r="F8" s="6" t="n">
         <v>3.46</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" s="8" t="n">
         <v>20.22</v>
       </c>
-      <c r="H8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" s="12" t="n">
-        <v>20.22</v>
+      <c r="I8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -717,23 +662,17 @@
       <c r="F9" s="6" t="n">
         <v>3.57</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" s="8" t="n">
         <v>15.84</v>
       </c>
-      <c r="H9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K9" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>15.84</v>
+      <c r="I9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -755,23 +694,17 @@
       <c r="F10" s="6" t="n">
         <v>3.19</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="G10" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="H10" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K10" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>20</v>
+      <c r="I10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -793,23 +726,17 @@
       <c r="F11" s="6" t="n">
         <v>3.15</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" s="8" t="n">
         <v>22.9</v>
       </c>
-      <c r="H11" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>22.9</v>
+      <c r="I11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -831,23 +758,17 @@
       <c r="F12" s="6" t="n">
         <v>3.44</v>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="G12" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" s="8" t="n">
         <v>18.3</v>
       </c>
-      <c r="H12" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K12" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>18.3</v>
+      <c r="I12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -869,23 +790,17 @@
       <c r="F13" s="6" t="n">
         <v>3.44</v>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="G13" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" s="8" t="n">
         <v>18.9</v>
       </c>
-      <c r="H13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>18.9</v>
+      <c r="I13" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -907,23 +822,17 @@
       <c r="F14" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="G14" s="7" t="n">
+      <c r="G14" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" s="8" t="n">
         <v>17.4</v>
       </c>
-      <c r="H14" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K14" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>17.4</v>
+      <c r="I14" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -945,23 +854,17 @@
       <c r="F15" s="6" t="n">
         <v>3.73</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="8" t="n">
         <v>17.6</v>
       </c>
-      <c r="H15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>17.6</v>
+      <c r="I15" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -983,23 +886,17 @@
       <c r="F16" s="6" t="n">
         <v>3.78</v>
       </c>
-      <c r="G16" s="7" t="n">
+      <c r="G16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="H16" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K16" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>18</v>
+      <c r="I16" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -1021,23 +918,17 @@
       <c r="F17" s="6" t="n">
         <v>5.25</v>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G17" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" s="8" t="n">
         <v>17.98</v>
       </c>
-      <c r="H17" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I17" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K17" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>17.98</v>
+      <c r="I17" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="18">
@@ -1059,23 +950,17 @@
       <c r="F18" s="6" t="n">
         <v>5.424</v>
       </c>
-      <c r="G18" s="7" t="n">
+      <c r="G18" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H18" s="8" t="n">
         <v>17.82</v>
       </c>
-      <c r="H18" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I18" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K18" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>17.82</v>
+      <c r="I18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="19">
@@ -1097,23 +982,17 @@
       <c r="F19" s="6" t="n">
         <v>5.345</v>
       </c>
-      <c r="G19" s="7" t="n">
+      <c r="G19" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" s="8" t="n">
         <v>17.42</v>
       </c>
-      <c r="H19" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I19" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K19" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L19" s="12" t="n">
-        <v>17.42</v>
+      <c r="I19" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="20">
@@ -1135,23 +1014,17 @@
       <c r="F20" s="6" t="n">
         <v>2.2</v>
       </c>
-      <c r="G20" s="7" t="n">
+      <c r="G20" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" s="8" t="n">
         <v>19.47</v>
       </c>
-      <c r="H20" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I20" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="12" t="n">
-        <v>19.47</v>
+      <c r="I20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="21">
@@ -1173,23 +1046,17 @@
       <c r="F21" s="6" t="n">
         <v>1.615</v>
       </c>
-      <c r="G21" s="7" t="n">
+      <c r="G21" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H21" s="8" t="n">
         <v>18.52</v>
       </c>
-      <c r="H21" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I21" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K21" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>18.52</v>
+      <c r="I21" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -1211,23 +1078,17 @@
       <c r="F22" s="6" t="n">
         <v>1.835</v>
       </c>
-      <c r="G22" s="7" t="n">
+      <c r="G22" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H22" s="8" t="n">
         <v>19.9</v>
       </c>
-      <c r="H22" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I22" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>19.9</v>
+      <c r="I22" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="23">
@@ -1249,23 +1110,17 @@
       <c r="F23" s="6" t="n">
         <v>2.465</v>
       </c>
-      <c r="G23" s="7" t="n">
+      <c r="G23" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" s="8" t="n">
         <v>20.01</v>
       </c>
-      <c r="H23" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K23" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>20.01</v>
+      <c r="I23" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="24">
@@ -1287,23 +1142,17 @@
       <c r="F24" s="6" t="n">
         <v>3.52</v>
       </c>
-      <c r="G24" s="7" t="n">
+      <c r="G24" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H24" s="8" t="n">
         <v>16.87</v>
       </c>
-      <c r="H24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K24" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>16.87</v>
+      <c r="I24" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="25">
@@ -1325,23 +1174,17 @@
       <c r="F25" s="6" t="n">
         <v>3.435</v>
       </c>
-      <c r="G25" s="7" t="n">
+      <c r="G25" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H25" s="8" t="n">
         <v>17.3</v>
       </c>
-      <c r="H25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I25" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K25" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L25" s="12" t="n">
-        <v>17.3</v>
+      <c r="I25" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="26">
@@ -1363,23 +1206,17 @@
       <c r="F26" s="6" t="n">
         <v>3.84</v>
       </c>
-      <c r="G26" s="7" t="n">
+      <c r="G26" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" s="8" t="n">
         <v>15.41</v>
       </c>
-      <c r="H26" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I26" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K26" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L26" s="12" t="n">
-        <v>15.41</v>
+      <c r="I26" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="27">
@@ -1401,23 +1238,17 @@
       <c r="F27" s="6" t="n">
         <v>3.845</v>
       </c>
-      <c r="G27" s="7" t="n">
+      <c r="G27" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H27" s="8" t="n">
         <v>17.05</v>
       </c>
-      <c r="H27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I27" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K27" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L27" s="12" t="n">
-        <v>17.05</v>
+      <c r="I27" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="28">
@@ -1439,23 +1270,17 @@
       <c r="F28" s="6" t="n">
         <v>1.935</v>
       </c>
-      <c r="G28" s="7" t="n">
+      <c r="G28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H28" s="8" t="n">
         <v>18.9</v>
       </c>
-      <c r="H28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I28" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J28" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K28" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L28" s="12" t="n">
-        <v>18.9</v>
+      <c r="I28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="29">
@@ -1477,23 +1302,17 @@
       <c r="F29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="G29" s="7" t="n">
+      <c r="G29" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H29" s="8" t="n">
         <v>16.7</v>
       </c>
-      <c r="H29" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J29" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K29" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L29" s="12" t="n">
-        <v>16.7</v>
+      <c r="I29" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="30">
@@ -1515,23 +1334,17 @@
       <c r="F30" s="6" t="n">
         <v>1.513</v>
       </c>
-      <c r="G30" s="7" t="n">
+      <c r="G30" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H30" s="8" t="n">
         <v>16.9</v>
       </c>
-      <c r="H30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I30" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K30" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L30" s="12" t="n">
-        <v>16.9</v>
+      <c r="I30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J30" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="31">
@@ -1553,23 +1366,17 @@
       <c r="F31" s="6" t="n">
         <v>3.17</v>
       </c>
-      <c r="G31" s="7" t="n">
+      <c r="G31" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H31" s="8" t="n">
         <v>14.5</v>
       </c>
-      <c r="H31" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I31" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K31" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L31" s="12" t="n">
-        <v>14.5</v>
+      <c r="I31" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="32">
@@ -1591,23 +1398,17 @@
       <c r="F32" s="6" t="n">
         <v>2.77</v>
       </c>
-      <c r="G32" s="7" t="n">
+      <c r="G32" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H32" s="8" t="n">
         <v>15.5</v>
       </c>
-      <c r="H32" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I32" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J32" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K32" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="L32" s="12" t="n">
-        <v>15.5</v>
+      <c r="I32" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J32" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="33">
@@ -1629,23 +1430,17 @@
       <c r="F33" s="6" t="n">
         <v>3.57</v>
       </c>
-      <c r="G33" s="7" t="n">
+      <c r="G33" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H33" s="8" t="n">
         <v>14.6</v>
       </c>
-      <c r="H33" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I33" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K33" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L33" s="12" t="n">
-        <v>14.6</v>
+      <c r="I33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J33" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -1667,23 +1462,17 @@
       <c r="F34" s="6" t="n">
         <v>2.78</v>
       </c>
-      <c r="G34" s="7" t="n">
+      <c r="G34" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H34" s="8" t="n">
         <v>18.6</v>
       </c>
-      <c r="H34" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I34" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J34" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K34" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L34" s="12" t="n">
-        <v>18.6</v>
+      <c r="I34" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J34" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="35">
@@ -1695,10 +1484,8 @@
       <c r="F35" s="6"/>
       <c r="G35" s="7"/>
       <c r="H35" s="8"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="11"/>
-      <c r="L35" s="12"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fixed conflicts for final merge with main.
</commit_message>
<xml_diff>
--- a/tests/testthat/_output_excel_snaps/data_to_worksheet.xlsx
+++ b/tests/testthat/_output_excel_snaps/data_to_worksheet.xlsx
@@ -12,63 +12,62 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
-    <t xml:space="preserve">mpg</t>
+    <t xml:space="preserve">test_r_numeric</t>
   </si>
   <si>
-    <t xml:space="preserve">cyl</t>
+    <t xml:space="preserve">test_r_integer</t>
   </si>
   <si>
-    <t xml:space="preserve">disp</t>
+    <t xml:space="preserve">test_xlr_numeric</t>
   </si>
   <si>
-    <t xml:space="preserve">hp</t>
+    <t xml:space="preserve">test_xlr_vector</t>
   </si>
   <si>
-    <t xml:space="preserve">drat</t>
+    <t xml:space="preserve">test_xlr_numeric.1</t>
   </si>
   <si>
-    <t xml:space="preserve">wt</t>
+    <t xml:space="preserve">test_xlr_percent</t>
   </si>
   <si>
-    <t xml:space="preserve">qsec</t>
+    <t xml:space="preserve">test_r_char</t>
   </si>
   <si>
-    <t xml:space="preserve">vs</t>
+    <t xml:space="preserve">test_xlr_scientific</t>
   </si>
   <si>
-    <t xml:space="preserve">am</t>
+    <t xml:space="preserve">test_r_factor</t>
   </si>
   <si>
-    <t xml:space="preserve">gear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">scientific</t>
+    <t xml:space="preserve">test_r_complex</t>
   </si>
   <si>
     <t xml:space="preserve">test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1+1i</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="11">
+  <numFmts count="7">
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="0"/>
     <numFmt numFmtId="168" formatCode="0.00"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
     <numFmt numFmtId="170" formatCode="0.00%"/>
-    <numFmt numFmtId="171" formatCode="0.00"/>
-    <numFmt numFmtId="172" formatCode="0.00"/>
-    <numFmt numFmtId="173" formatCode="0.00"/>
-    <numFmt numFmtId="174" formatCode="0.00"/>
-    <numFmt numFmtId="175" formatCode="0.00E+00"/>
+    <numFmt numFmtId="171" formatCode="0.00E+00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -104,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -124,22 +123,10 @@
     <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="172" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="173" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="174" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="175" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -463,12 +450,6 @@
       <c r="J2" t="s">
         <v>9</v>
       </c>
-      <c r="K2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L2" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -489,23 +470,17 @@
       <c r="F3" s="6" t="n">
         <v>2.62</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="G3" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="8" t="n">
         <v>16.46</v>
       </c>
-      <c r="H3" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K3" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>16.46</v>
+      <c r="I3" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -527,23 +502,17 @@
       <c r="F4" s="6" t="n">
         <v>2.875</v>
       </c>
-      <c r="G4" s="7" t="n">
+      <c r="G4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="8" t="n">
         <v>17.02</v>
       </c>
-      <c r="H4" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K4" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>17.02</v>
+      <c r="I4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -565,23 +534,17 @@
       <c r="F5" s="6" t="n">
         <v>2.32</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="8" t="n">
         <v>18.61</v>
       </c>
-      <c r="H5" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>18.61</v>
+      <c r="I5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -603,23 +566,17 @@
       <c r="F6" s="6" t="n">
         <v>3.215</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="8" t="n">
         <v>19.44</v>
       </c>
-      <c r="H6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K6" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>19.44</v>
+      <c r="I6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -641,23 +598,17 @@
       <c r="F7" s="6" t="n">
         <v>3.44</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="8" t="n">
         <v>17.02</v>
       </c>
-      <c r="H7" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L7" s="12" t="n">
-        <v>17.02</v>
+      <c r="I7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -679,23 +630,17 @@
       <c r="F8" s="6" t="n">
         <v>3.46</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" s="8" t="n">
         <v>20.22</v>
       </c>
-      <c r="H8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" s="12" t="n">
-        <v>20.22</v>
+      <c r="I8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -717,23 +662,17 @@
       <c r="F9" s="6" t="n">
         <v>3.57</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" s="8" t="n">
         <v>15.84</v>
       </c>
-      <c r="H9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K9" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>15.84</v>
+      <c r="I9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -755,23 +694,17 @@
       <c r="F10" s="6" t="n">
         <v>3.19</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="G10" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="H10" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K10" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>20</v>
+      <c r="I10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -793,23 +726,17 @@
       <c r="F11" s="6" t="n">
         <v>3.15</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" s="8" t="n">
         <v>22.9</v>
       </c>
-      <c r="H11" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>22.9</v>
+      <c r="I11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -831,23 +758,17 @@
       <c r="F12" s="6" t="n">
         <v>3.44</v>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="G12" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" s="8" t="n">
         <v>18.3</v>
       </c>
-      <c r="H12" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K12" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>18.3</v>
+      <c r="I12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -869,23 +790,17 @@
       <c r="F13" s="6" t="n">
         <v>3.44</v>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="G13" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" s="8" t="n">
         <v>18.9</v>
       </c>
-      <c r="H13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>18.9</v>
+      <c r="I13" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -907,23 +822,17 @@
       <c r="F14" s="6" t="n">
         <v>4.07</v>
       </c>
-      <c r="G14" s="7" t="n">
+      <c r="G14" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" s="8" t="n">
         <v>17.4</v>
       </c>
-      <c r="H14" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I14" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K14" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>17.4</v>
+      <c r="I14" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -945,23 +854,17 @@
       <c r="F15" s="6" t="n">
         <v>3.73</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="8" t="n">
         <v>17.6</v>
       </c>
-      <c r="H15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>17.6</v>
+      <c r="I15" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -983,23 +886,17 @@
       <c r="F16" s="6" t="n">
         <v>3.78</v>
       </c>
-      <c r="G16" s="7" t="n">
+      <c r="G16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="H16" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K16" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>18</v>
+      <c r="I16" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -1021,23 +918,17 @@
       <c r="F17" s="6" t="n">
         <v>5.25</v>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G17" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" s="8" t="n">
         <v>17.98</v>
       </c>
-      <c r="H17" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I17" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K17" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>17.98</v>
+      <c r="I17" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="18">
@@ -1059,23 +950,17 @@
       <c r="F18" s="6" t="n">
         <v>5.424</v>
       </c>
-      <c r="G18" s="7" t="n">
+      <c r="G18" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H18" s="8" t="n">
         <v>17.82</v>
       </c>
-      <c r="H18" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I18" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K18" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>17.82</v>
+      <c r="I18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="19">
@@ -1097,23 +982,17 @@
       <c r="F19" s="6" t="n">
         <v>5.345</v>
       </c>
-      <c r="G19" s="7" t="n">
+      <c r="G19" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" s="8" t="n">
         <v>17.42</v>
       </c>
-      <c r="H19" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I19" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K19" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L19" s="12" t="n">
-        <v>17.42</v>
+      <c r="I19" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="20">
@@ -1135,23 +1014,17 @@
       <c r="F20" s="6" t="n">
         <v>2.2</v>
       </c>
-      <c r="G20" s="7" t="n">
+      <c r="G20" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" s="8" t="n">
         <v>19.47</v>
       </c>
-      <c r="H20" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I20" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="12" t="n">
-        <v>19.47</v>
+      <c r="I20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="21">
@@ -1173,23 +1046,17 @@
       <c r="F21" s="6" t="n">
         <v>1.615</v>
       </c>
-      <c r="G21" s="7" t="n">
+      <c r="G21" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H21" s="8" t="n">
         <v>18.52</v>
       </c>
-      <c r="H21" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I21" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K21" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>18.52</v>
+      <c r="I21" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -1211,23 +1078,17 @@
       <c r="F22" s="6" t="n">
         <v>1.835</v>
       </c>
-      <c r="G22" s="7" t="n">
+      <c r="G22" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H22" s="8" t="n">
         <v>19.9</v>
       </c>
-      <c r="H22" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I22" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>19.9</v>
+      <c r="I22" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="23">
@@ -1249,23 +1110,17 @@
       <c r="F23" s="6" t="n">
         <v>2.465</v>
       </c>
-      <c r="G23" s="7" t="n">
+      <c r="G23" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" s="8" t="n">
         <v>20.01</v>
       </c>
-      <c r="H23" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K23" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>20.01</v>
+      <c r="I23" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="24">
@@ -1287,23 +1142,17 @@
       <c r="F24" s="6" t="n">
         <v>3.52</v>
       </c>
-      <c r="G24" s="7" t="n">
+      <c r="G24" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H24" s="8" t="n">
         <v>16.87</v>
       </c>
-      <c r="H24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K24" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>16.87</v>
+      <c r="I24" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="25">
@@ -1325,23 +1174,17 @@
       <c r="F25" s="6" t="n">
         <v>3.435</v>
       </c>
-      <c r="G25" s="7" t="n">
+      <c r="G25" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H25" s="8" t="n">
         <v>17.3</v>
       </c>
-      <c r="H25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I25" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K25" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L25" s="12" t="n">
-        <v>17.3</v>
+      <c r="I25" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="26">
@@ -1363,23 +1206,17 @@
       <c r="F26" s="6" t="n">
         <v>3.84</v>
       </c>
-      <c r="G26" s="7" t="n">
+      <c r="G26" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" s="8" t="n">
         <v>15.41</v>
       </c>
-      <c r="H26" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I26" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K26" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L26" s="12" t="n">
-        <v>15.41</v>
+      <c r="I26" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="27">
@@ -1401,23 +1238,17 @@
       <c r="F27" s="6" t="n">
         <v>3.845</v>
       </c>
-      <c r="G27" s="7" t="n">
+      <c r="G27" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H27" s="8" t="n">
         <v>17.05</v>
       </c>
-      <c r="H27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I27" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K27" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L27" s="12" t="n">
-        <v>17.05</v>
+      <c r="I27" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="28">
@@ -1439,23 +1270,17 @@
       <c r="F28" s="6" t="n">
         <v>1.935</v>
       </c>
-      <c r="G28" s="7" t="n">
+      <c r="G28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H28" s="8" t="n">
         <v>18.9</v>
       </c>
-      <c r="H28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I28" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J28" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K28" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L28" s="12" t="n">
-        <v>18.9</v>
+      <c r="I28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="29">
@@ -1477,23 +1302,17 @@
       <c r="F29" s="6" t="n">
         <v>2.14</v>
       </c>
-      <c r="G29" s="7" t="n">
+      <c r="G29" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H29" s="8" t="n">
         <v>16.7</v>
       </c>
-      <c r="H29" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J29" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K29" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L29" s="12" t="n">
-        <v>16.7</v>
+      <c r="I29" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="30">
@@ -1515,23 +1334,17 @@
       <c r="F30" s="6" t="n">
         <v>1.513</v>
       </c>
-      <c r="G30" s="7" t="n">
+      <c r="G30" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H30" s="8" t="n">
         <v>16.9</v>
       </c>
-      <c r="H30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I30" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K30" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L30" s="12" t="n">
-        <v>16.9</v>
+      <c r="I30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J30" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="31">
@@ -1553,23 +1366,17 @@
       <c r="F31" s="6" t="n">
         <v>3.17</v>
       </c>
-      <c r="G31" s="7" t="n">
+      <c r="G31" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H31" s="8" t="n">
         <v>14.5</v>
       </c>
-      <c r="H31" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I31" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K31" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L31" s="12" t="n">
-        <v>14.5</v>
+      <c r="I31" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="32">
@@ -1591,23 +1398,17 @@
       <c r="F32" s="6" t="n">
         <v>2.77</v>
       </c>
-      <c r="G32" s="7" t="n">
+      <c r="G32" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H32" s="8" t="n">
         <v>15.5</v>
       </c>
-      <c r="H32" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I32" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J32" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K32" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="L32" s="12" t="n">
-        <v>15.5</v>
+      <c r="I32" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J32" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="33">
@@ -1629,23 +1430,17 @@
       <c r="F33" s="6" t="n">
         <v>3.57</v>
       </c>
-      <c r="G33" s="7" t="n">
+      <c r="G33" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H33" s="8" t="n">
         <v>14.6</v>
       </c>
-      <c r="H33" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I33" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="K33" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L33" s="12" t="n">
-        <v>14.6</v>
+      <c r="I33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J33" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -1667,23 +1462,17 @@
       <c r="F34" s="6" t="n">
         <v>2.78</v>
       </c>
-      <c r="G34" s="7" t="n">
+      <c r="G34" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H34" s="8" t="n">
         <v>18.6</v>
       </c>
-      <c r="H34" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I34" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J34" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="K34" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L34" s="12" t="n">
-        <v>18.6</v>
+      <c r="I34" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J34" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="35">
@@ -1695,10 +1484,8 @@
       <c r="F35" s="6"/>
       <c r="G35" s="7"/>
       <c r="H35" s="8"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="11"/>
-      <c r="L35" s="12"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>